<commit_message>
Fixed set current parsing
</commit_message>
<xml_diff>
--- a/Electrical/5_07/Pulsing_Analysis_Results.xlsx
+++ b/Electrical/5_07/Pulsing_Analysis_Results.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="32" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="56" uniqueCount="11">
   <si>
     <t>Filename</t>
   </si>
@@ -40,6 +40,12 @@
   </si>
   <si>
     <t>1khz_10%_2_5mA_dummy.csv</t>
+  </si>
+  <si>
+    <t>1khz_10%_3mA_dummy.csv</t>
+  </si>
+  <si>
+    <t>1khz_10%_2.5mA_dummy.csv</t>
   </si>
 </sst>
 </file>
@@ -122,7 +128,7 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B2" s="0">
         <v>1000</v>

</xml_diff>